<commit_message>
Execution all models withot P and Plag
</commit_message>
<xml_diff>
--- a/results/cross_validation/global/metrics_summary.xlsx
+++ b/results/cross_validation/global/metrics_summary.xlsx
@@ -482,25 +482,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7731888835334902</v>
+        <v>0.1976663776707422</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8725112218547966</v>
+        <v>0.2834899052365473</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9831207109723542</v>
+        <v>0.3544706790577623</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9027960099415565</v>
+        <v>-1.348275342440982</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8957367555224912</v>
+        <v>0.7756189814622407</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8870421897632809</v>
+        <v>0.5263922246879603</v>
       </c>
       <c r="H2" t="n">
-        <v>0.885732628597995</v>
+        <v>0.1315604709457118</v>
       </c>
     </row>
     <row r="3">
@@ -510,25 +510,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.137344214703369</v>
+        <v>0.3312790716453166</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1014033310516529</v>
+        <v>0.2334488868229029</v>
       </c>
       <c r="D3" t="n">
-        <v>0.005609288257706873</v>
+        <v>0.0758037974624562</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01296072863041777</v>
+        <v>0.09252231678204231</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03377388732444474</v>
+        <v>0.07600437648687226</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0361330391110217</v>
+        <v>0.1083351994284809</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0545374148464355</v>
+        <v>0.1528989414380119</v>
       </c>
     </row>
     <row r="4">
@@ -538,25 +538,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1056178896671258</v>
+        <v>0.3736183010761268</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05064126661183183</v>
+        <v>0.2846131186358859</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0002215835106912817</v>
+        <v>0.008474210788989019</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0006536415402608362</v>
+        <v>0.01579081590032257</v>
       </c>
       <c r="F4" t="n">
-        <v>0.004431567486978748</v>
+        <v>0.009537010203644758</v>
       </c>
       <c r="G4" t="n">
-        <v>0.004265919030053162</v>
+        <v>0.01788607992002319</v>
       </c>
       <c r="H4" t="n">
-        <v>0.02763864464115695</v>
+        <v>0.1183199227541654</v>
       </c>
     </row>
     <row r="5">
@@ -566,25 +566,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3249890608422471</v>
+        <v>0.6112432421517041</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2250361451230265</v>
+        <v>0.5334914419518704</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01488568139828613</v>
+        <v>0.09205547669198731</v>
       </c>
       <c r="E5" t="n">
-        <v>0.02556641430198682</v>
+        <v>0.1256615132024224</v>
       </c>
       <c r="F5" t="n">
-        <v>0.06657001943051202</v>
+        <v>0.0976576172330902</v>
       </c>
       <c r="G5" t="n">
-        <v>0.06531400332281863</v>
+        <v>0.1337388497035293</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1203935540698129</v>
+        <v>0.2656413568224339</v>
       </c>
     </row>
     <row r="6">
@@ -594,25 +594,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>27.93408076496081</v>
+        <v>57.47912594050217</v>
       </c>
       <c r="C6" t="n">
-        <v>29.80296874871599</v>
+        <v>46.74812787068655</v>
       </c>
       <c r="D6" t="n">
-        <v>8.764258404308217</v>
+        <v>83.73984386171685</v>
       </c>
       <c r="E6" t="n">
-        <v>31.57536297007722</v>
+        <v>161.7018281472745</v>
       </c>
       <c r="F6" t="n">
-        <v>19.76093796416055</v>
+        <v>45.13625242061012</v>
       </c>
       <c r="G6" t="n">
-        <v>26.95523531728998</v>
+        <v>94.84539752853622</v>
       </c>
       <c r="H6" t="n">
-        <v>24.13214069491879</v>
+        <v>81.60842929488773</v>
       </c>
     </row>
     <row r="7">
@@ -622,25 +622,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.142975857706941</v>
+        <v>0.5042328974520661</v>
       </c>
       <c r="C7" t="n">
-        <v>0.07469552007184332</v>
+        <v>0.416182211474156</v>
       </c>
       <c r="D7" t="n">
-        <v>0.006218895165777636</v>
+        <v>0.2015907438349636</v>
       </c>
       <c r="E7" t="n">
-        <v>0.03061874609571564</v>
+        <v>1.435072347725041</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03538107058413777</v>
+        <v>0.07599021270387912</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03787348639205296</v>
+        <v>0.1566025885376282</v>
       </c>
       <c r="H7" t="n">
-        <v>0.05462726266941139</v>
+        <v>0.4649451669546223</v>
       </c>
     </row>
     <row r="8">
@@ -650,25 +650,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-34.21476770963743</v>
+        <v>-8.736849997315936</v>
       </c>
       <c r="C8" t="n">
-        <v>-40.74482734065539</v>
+        <v>-10.84936749088962</v>
       </c>
       <c r="D8" t="n">
-        <v>-172.7089313380501</v>
+        <v>-92.18528279819398</v>
       </c>
       <c r="E8" t="n">
-        <v>-149.9919806672965</v>
+        <v>-79.11486238178162</v>
       </c>
       <c r="F8" t="n">
-        <v>-142.3130519203876</v>
+        <v>-117.6195314390963</v>
       </c>
       <c r="G8" t="n">
-        <v>-132.4274409852517</v>
+        <v>-92.59331316919014</v>
       </c>
       <c r="H8" t="n">
-        <v>-112.0668333268798</v>
+        <v>-66.84986787941126</v>
       </c>
     </row>
     <row r="9">
@@ -678,25 +678,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-32.548341021525</v>
+        <v>-5.403996621091071</v>
       </c>
       <c r="C9" t="n">
-        <v>-39.32872693845097</v>
+        <v>-8.017166686480779</v>
       </c>
       <c r="D9" t="n">
-        <v>-170.6198864626032</v>
+        <v>-88.00719304730029</v>
       </c>
       <c r="E9" t="n">
-        <v>-147.9029357918496</v>
+        <v>-74.93677263088793</v>
       </c>
       <c r="F9" t="n">
-        <v>-139.7213781883789</v>
+        <v>-112.436183975079</v>
       </c>
       <c r="G9" t="n">
-        <v>-129.9896893355153</v>
+        <v>-87.71780986971734</v>
       </c>
       <c r="H9" t="n">
-        <v>-110.0184929563872</v>
+        <v>-62.75318713842606</v>
       </c>
     </row>
   </sheetData>
@@ -757,25 +757,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6121564601983727</v>
+        <v>0.8993423560191121</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8698955032248902</v>
+        <v>0.4704503519994442</v>
       </c>
       <c r="D2" t="n">
-        <v>0.977451133537302</v>
+        <v>-0.3143669507920797</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9461970375981978</v>
+        <v>0.6389779037375329</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9214353229687969</v>
+        <v>0.255343219810068</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8987935181479894</v>
+        <v>-3.419031327115063</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8709881626125915</v>
+        <v>-0.244880741056831</v>
       </c>
     </row>
     <row r="3">
@@ -785,25 +785,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1689854375460691</v>
+        <v>0.1899207933408533</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1113839974738382</v>
+        <v>0.2039762243061733</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01300915847487365</v>
+        <v>0.1256851547415206</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01274105594382345</v>
+        <v>0.03292652375455817</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0373319157115065</v>
+        <v>0.1251701488618647</v>
       </c>
       <c r="G3" t="n">
-        <v>0.02666956452588106</v>
+        <v>0.3079648122218118</v>
       </c>
       <c r="H3" t="n">
-        <v>0.06168685494599866</v>
+        <v>0.1642739428711303</v>
       </c>
     </row>
     <row r="4">
@@ -813,25 +813,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1806049757747402</v>
+        <v>0.04687269346295922</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05168028593922516</v>
+        <v>0.2103484345740183</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0002960111047763965</v>
+        <v>0.01725440229242429</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0003617943172267443</v>
+        <v>0.002427668235916175</v>
       </c>
       <c r="F4" t="n">
-        <v>0.003339284808382977</v>
+        <v>0.03165062426922503</v>
       </c>
       <c r="G4" t="n">
-        <v>0.003822123109437519</v>
+        <v>0.1668873519523422</v>
       </c>
       <c r="H4" t="n">
-        <v>0.04001741250896484</v>
+        <v>0.0792401957978142</v>
       </c>
     </row>
     <row r="5">
@@ -841,25 +841,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4249764414349814</v>
+        <v>0.2165010241614557</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2273329847145485</v>
+        <v>0.4586375852173678</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01720497325706717</v>
+        <v>0.1313560135373493</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0190208915991534</v>
+        <v>0.04927137339182028</v>
       </c>
       <c r="F5" t="n">
-        <v>0.05778654521930669</v>
+        <v>0.1779062232447899</v>
       </c>
       <c r="G5" t="n">
-        <v>0.06182332172762572</v>
+        <v>0.4085184842235932</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1346908596587805</v>
+        <v>0.2403651172960627</v>
       </c>
     </row>
     <row r="6">
@@ -869,25 +869,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>26.86905887367338</v>
+        <v>49.13274132115505</v>
       </c>
       <c r="C6" t="n">
-        <v>29.72821302799129</v>
+        <v>42.63571246132688</v>
       </c>
       <c r="D6" t="n">
-        <v>10.63193795583293</v>
+        <v>64.5007419751291</v>
       </c>
       <c r="E6" t="n">
-        <v>14.8265130339079</v>
+        <v>46.09915640913847</v>
       </c>
       <c r="F6" t="n">
-        <v>21.61918230398741</v>
+        <v>61.55702471844994</v>
       </c>
       <c r="G6" t="n">
-        <v>14.44268565383375</v>
+        <v>250.7010664415048</v>
       </c>
       <c r="H6" t="n">
-        <v>19.68626514153778</v>
+        <v>85.77107388778404</v>
       </c>
     </row>
     <row r="7">
@@ -897,25 +897,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.2462765449828064</v>
+        <v>0.06700817861833784</v>
       </c>
       <c r="C7" t="n">
-        <v>0.07870754918999057</v>
+        <v>0.3101087986019796</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01047186771215289</v>
+        <v>0.8207763336846419</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01989414474259937</v>
+        <v>0.1140059966438815</v>
       </c>
       <c r="F7" t="n">
-        <v>0.029406902475229</v>
+        <v>0.2495524710454372</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03653743073220946</v>
+        <v>2.893061089002317</v>
       </c>
       <c r="H7" t="n">
-        <v>0.07021573997249794</v>
+        <v>0.7424188112660991</v>
       </c>
     </row>
     <row r="8">
@@ -925,25 +925,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-15.09453247940176</v>
+        <v>-36.02544003443792</v>
       </c>
       <c r="C8" t="n">
-        <v>-30.4401832996503</v>
+        <v>-7.384848664690882</v>
       </c>
       <c r="D8" t="n">
-        <v>-156.6273853523565</v>
+        <v>-69.25344721682991</v>
       </c>
       <c r="E8" t="n">
-        <v>-152.4131285335323</v>
+        <v>-110.4373051762583</v>
       </c>
       <c r="F8" t="n">
-        <v>-139.9539628520262</v>
+        <v>-77.23092997388916</v>
       </c>
       <c r="G8" t="n">
-        <v>-125.1737305736407</v>
+        <v>-28.76090583442107</v>
       </c>
       <c r="H8" t="n">
-        <v>-103.2838205151013</v>
+        <v>-54.84881281675453</v>
       </c>
     </row>
     <row r="9">
@@ -953,25 +953,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-9.262039071008246</v>
+        <v>-29.35973328198819</v>
       </c>
       <c r="C9" t="n">
-        <v>-25.48383189193483</v>
+        <v>-1.720447055873201</v>
       </c>
       <c r="D9" t="n">
-        <v>-149.3157282882925</v>
+        <v>-60.89726771504253</v>
       </c>
       <c r="E9" t="n">
-        <v>-145.1014714694684</v>
+        <v>-102.0811256744709</v>
       </c>
       <c r="F9" t="n">
-        <v>-130.8831047899959</v>
+        <v>-66.86423504585453</v>
       </c>
       <c r="G9" t="n">
-        <v>-116.6415997995633</v>
+        <v>-19.00989923547546</v>
       </c>
       <c r="H9" t="n">
-        <v>-96.11462921837717</v>
+        <v>-46.65545133478414</v>
       </c>
     </row>
   </sheetData>
@@ -1032,25 +1032,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9322547539081764</v>
+        <v>0.8688950948458743</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8707490903463868</v>
+        <v>0.9184098962007062</v>
       </c>
       <c r="D2" t="n">
-        <v>0.886701103291085</v>
+        <v>0.7639331374052144</v>
       </c>
       <c r="E2" t="n">
-        <v>0.875492042273109</v>
+        <v>0.8701651020985333</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9169156346243755</v>
+        <v>0.9223722895751213</v>
       </c>
       <c r="G2" t="n">
-        <v>0.873101387393599</v>
+        <v>0.7290193634425375</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8925356686394553</v>
+        <v>0.8454658139279978</v>
       </c>
     </row>
     <row r="3">
@@ -1060,25 +1060,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.08057855596760877</v>
+        <v>0.1174371246339853</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1018966926052491</v>
+        <v>0.08063647277549375</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01806707805812173</v>
+        <v>0.02609243649317531</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01358435692549985</v>
+        <v>0.01317981080501577</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03421539133747273</v>
+        <v>0.03297359540111087</v>
       </c>
       <c r="G3" t="n">
-        <v>0.04145526427771951</v>
+        <v>0.05177196471575596</v>
       </c>
       <c r="H3" t="n">
-        <v>0.04829955652861195</v>
+        <v>0.05368190080408949</v>
       </c>
     </row>
     <row r="4">
@@ -1088,25 +1088,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.03154655749977325</v>
+        <v>0.06105090272077578</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05134122289677524</v>
+        <v>0.03240933248792397</v>
       </c>
       <c r="D4" t="n">
-        <v>0.001487335589140733</v>
+        <v>0.003098976745167125</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0008372451914206881</v>
+        <v>0.0008730658339528877</v>
       </c>
       <c r="F4" t="n">
-        <v>0.003531388018088249</v>
+        <v>0.003299460316350529</v>
       </c>
       <c r="G4" t="n">
-        <v>0.004792401740707764</v>
+        <v>0.01023374525270873</v>
       </c>
       <c r="H4" t="n">
-        <v>0.01558935848931765</v>
+        <v>0.01849424722614651</v>
       </c>
     </row>
     <row r="5">
@@ -1116,25 +1116,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1776135059610424</v>
+        <v>0.2470848087616391</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2265860165517176</v>
+        <v>0.1800259217110802</v>
       </c>
       <c r="D5" t="n">
-        <v>0.03856599005783117</v>
+        <v>0.05566845377022003</v>
       </c>
       <c r="E5" t="n">
-        <v>0.02893518950034176</v>
+        <v>0.02954768745524576</v>
       </c>
       <c r="F5" t="n">
-        <v>0.05942548290159912</v>
+        <v>0.05744092893008024</v>
       </c>
       <c r="G5" t="n">
-        <v>0.06922717487163378</v>
+        <v>0.1011619753302037</v>
       </c>
       <c r="H5" t="n">
-        <v>0.100058893307361</v>
+        <v>0.1118216293264115</v>
       </c>
     </row>
     <row r="6">
@@ -1144,25 +1144,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20.498398824979</v>
+        <v>26.37741035006173</v>
       </c>
       <c r="C6" t="n">
-        <v>24.00269452055293</v>
+        <v>24.26671134951604</v>
       </c>
       <c r="D6" t="n">
-        <v>30.40051159010692</v>
+        <v>42.49977455893399</v>
       </c>
       <c r="E6" t="n">
-        <v>26.54890738708907</v>
+        <v>23.99208358450983</v>
       </c>
       <c r="F6" t="n">
-        <v>20.25531126558197</v>
+        <v>22.58422612572181</v>
       </c>
       <c r="G6" t="n">
-        <v>29.37057757740349</v>
+        <v>38.28069000917452</v>
       </c>
       <c r="H6" t="n">
-        <v>25.17940019428556</v>
+        <v>29.66681599631965</v>
       </c>
     </row>
     <row r="7">
@@ -1172,25 +1172,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.04590616407738837</v>
+        <v>0.08506710345078075</v>
       </c>
       <c r="C7" t="n">
-        <v>0.07821412892382662</v>
+        <v>0.05016356388133492</v>
       </c>
       <c r="D7" t="n">
-        <v>0.03853080392507303</v>
+        <v>0.07598934250005268</v>
       </c>
       <c r="E7" t="n">
-        <v>0.04143845895206181</v>
+        <v>0.04256161545420705</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03089728122534912</v>
+        <v>0.02859793534890898</v>
       </c>
       <c r="G7" t="n">
-        <v>0.04492426500041575</v>
+        <v>0.09145781264413488</v>
       </c>
       <c r="H7" t="n">
-        <v>0.04665185035068578</v>
+        <v>0.0623062288799032</v>
       </c>
     </row>
     <row r="8">
@@ -1200,25 +1200,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-44.75694374407698</v>
+        <v>-35.53280396321205</v>
       </c>
       <c r="C8" t="n">
-        <v>-30.53891926377734</v>
+        <v>-39.43963286862898</v>
       </c>
       <c r="D8" t="n">
-        <v>-122.7261480542008</v>
+        <v>-109.3103493878705</v>
       </c>
       <c r="E8" t="n">
-        <v>-134.7932653817703</v>
+        <v>-135.9134914697214</v>
       </c>
       <c r="F8" t="n">
-        <v>-138.4437355347539</v>
+        <v>-142.2779018383612</v>
       </c>
       <c r="G8" t="n">
-        <v>-119.518089649401</v>
+        <v>-102.551616528988</v>
       </c>
       <c r="H8" t="n">
-        <v>-98.46285027133007</v>
+        <v>-94.17096600946371</v>
       </c>
     </row>
     <row r="9">
@@ -1228,25 +1228,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-38.92445033568347</v>
+        <v>-30.53352389887475</v>
       </c>
       <c r="C9" t="n">
-        <v>-25.58256785606187</v>
+        <v>-35.19133166201571</v>
       </c>
       <c r="D9" t="n">
-        <v>-115.4144909901369</v>
+        <v>-103.04321476153</v>
       </c>
       <c r="E9" t="n">
-        <v>-127.4816083177063</v>
+        <v>-129.6463568433809</v>
       </c>
       <c r="F9" t="n">
-        <v>-129.3728774727236</v>
+        <v>-134.5028806423352</v>
       </c>
       <c r="G9" t="n">
-        <v>-110.9859588753236</v>
+        <v>-95.2383615797788</v>
       </c>
       <c r="H9" t="n">
-        <v>-91.29365897460595</v>
+        <v>-88.02594489798589</v>
       </c>
     </row>
   </sheetData>
@@ -1582,25 +1582,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.3649808836908726</v>
+        <v>0.9312334534953024</v>
       </c>
       <c r="C2" t="n">
-        <v>0.006842187883637441</v>
+        <v>0.9361687079093279</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7361808303316463</v>
+        <v>0.9098130984259211</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8355718671592859</v>
+        <v>0.6085067670360935</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8898722665862924</v>
+        <v>0.6071193009776117</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.8353534731670564</v>
+        <v>-0.9285105797763178</v>
       </c>
       <c r="H2" t="n">
-        <v>0.333015760414113</v>
+        <v>0.5107217913446565</v>
       </c>
     </row>
     <row r="3">
@@ -1610,25 +1610,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2919943856347123</v>
+        <v>0.0800390014471514</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2965741852309667</v>
+        <v>0.06973092412027639</v>
       </c>
       <c r="D3" t="n">
-        <v>0.02306048540544114</v>
+        <v>0.01408566284576012</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01511410032868808</v>
+        <v>0.01777861365224019</v>
       </c>
       <c r="F3" t="n">
-        <v>0.05952263207637042</v>
+        <v>0.07930506973908301</v>
       </c>
       <c r="G3" t="n">
-        <v>0.185429179009242</v>
+        <v>0.154291098654353</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1452824946142368</v>
+        <v>0.06920506174314402</v>
       </c>
     </row>
     <row r="4">
@@ -1638,25 +1638,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2957058719507534</v>
+        <v>0.03202214086625183</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3945035028394818</v>
+        <v>0.02535515304146834</v>
       </c>
       <c r="D4" t="n">
-        <v>0.003463296215085071</v>
+        <v>0.001183931991236286</v>
       </c>
       <c r="E4" t="n">
-        <v>0.00110568566112973</v>
+        <v>0.002632569297231171</v>
       </c>
       <c r="F4" t="n">
-        <v>0.004680829617920888</v>
+        <v>0.01669886008990135</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0693132178434563</v>
+        <v>0.07283135149916661</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1281287340213046</v>
+        <v>0.0251206677975426</v>
       </c>
     </row>
     <row r="5">
@@ -1666,25 +1666,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5437884441129228</v>
+        <v>0.1789473131015155</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6280951383663799</v>
+        <v>0.159233014923</v>
       </c>
       <c r="D5" t="n">
-        <v>0.05884977667829395</v>
+        <v>0.03440831282170467</v>
       </c>
       <c r="E5" t="n">
-        <v>0.03325185199548635</v>
+        <v>0.05130856943270949</v>
       </c>
       <c r="F5" t="n">
-        <v>0.06841658876267427</v>
+        <v>0.1292240693133495</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2632740356424391</v>
+        <v>0.2698728432042887</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2659459725930327</v>
+        <v>0.1371656871327613</v>
       </c>
     </row>
     <row r="6">
@@ -1694,25 +1694,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>57.64472177160614</v>
+        <v>16.88309192410653</v>
       </c>
       <c r="C6" t="n">
-        <v>76.640841679392</v>
+        <v>20.11525247383939</v>
       </c>
       <c r="D6" t="n">
-        <v>28.74932697048213</v>
+        <v>18.49556494262038</v>
       </c>
       <c r="E6" t="n">
-        <v>34.21747731001079</v>
+        <v>34.30205163861444</v>
       </c>
       <c r="F6" t="n">
-        <v>35.898122408214</v>
+        <v>46.50810423900686</v>
       </c>
       <c r="G6" t="n">
-        <v>142.6644679421298</v>
+        <v>91.00086533547925</v>
       </c>
       <c r="H6" t="n">
-        <v>62.63582634697247</v>
+        <v>37.88415509227781</v>
       </c>
     </row>
     <row r="7">
@@ -1722,25 +1722,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.4014998452582656</v>
+        <v>0.04504546255778556</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5780997956225461</v>
+        <v>0.03889799475622946</v>
       </c>
       <c r="D7" t="n">
-        <v>0.08557005825106569</v>
+        <v>0.02988482286608909</v>
       </c>
       <c r="E7" t="n">
-        <v>0.05410241981500505</v>
+        <v>0.1212907683972338</v>
       </c>
       <c r="F7" t="n">
-        <v>0.04031490075665692</v>
+        <v>0.1315534117696475</v>
       </c>
       <c r="G7" t="n">
-        <v>1.206250588881073</v>
+        <v>1.263070239964624</v>
       </c>
       <c r="H7" t="n">
-        <v>0.3943062680974354</v>
+        <v>0.2716237833852682</v>
       </c>
     </row>
     <row r="8">
@@ -1750,25 +1750,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-4.712629906895394</v>
+        <v>-50.50257112722071</v>
       </c>
       <c r="C8" t="n">
-        <v>2.048091106778578</v>
+        <v>-47.12159940707654</v>
       </c>
       <c r="D8" t="n">
-        <v>-102.9762240818653</v>
+        <v>-133.5171978640897</v>
       </c>
       <c r="E8" t="n">
-        <v>-126.9530822013997</v>
+        <v>-116.7356948019295</v>
       </c>
       <c r="F8" t="n">
-        <v>-128.8355577313607</v>
+        <v>-102.4952001394291</v>
       </c>
       <c r="G8" t="n">
-        <v>-50.72799143254564</v>
+        <v>-57.49021910056435</v>
       </c>
       <c r="H8" t="n">
-        <v>-68.69289904121469</v>
+        <v>-84.64374707338497</v>
       </c>
     </row>
     <row r="9">
@@ -1778,25 +1778,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.953076845554335</v>
+        <v>-47.16971775099584</v>
       </c>
       <c r="C9" t="n">
-        <v>7.712492715596259</v>
+        <v>-44.2893986026677</v>
       </c>
       <c r="D9" t="n">
-        <v>-94.6200445800779</v>
+        <v>-129.339108113196</v>
       </c>
       <c r="E9" t="n">
-        <v>-118.5969026996123</v>
+        <v>-112.5576050510358</v>
       </c>
       <c r="F9" t="n">
-        <v>-118.4688628033261</v>
+        <v>-97.3118526754118</v>
       </c>
       <c r="G9" t="n">
-        <v>-40.97698483360003</v>
+        <v>-52.61471580109154</v>
       </c>
       <c r="H9" t="n">
-        <v>-60.49953755924429</v>
+        <v>-80.54706633239978</v>
       </c>
     </row>
   </sheetData>
@@ -1857,25 +1857,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7742858394957591</v>
+        <v>0.09889484127984349</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8522812276291934</v>
+        <v>0.1763499024048283</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9837499537097349</v>
+        <v>-0.2729382278028016</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9257703957739791</v>
+        <v>-4.827697156941836</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9036491499330408</v>
+        <v>0.4426369112681671</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8894622404613096</v>
+        <v>0.6402444639199151</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8881998011671696</v>
+        <v>-0.6237515443119807</v>
       </c>
     </row>
     <row r="3">
@@ -1885,25 +1885,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1371235456025501</v>
+        <v>0.3441535538509446</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1119640387571579</v>
+        <v>0.2548422155919852</v>
       </c>
       <c r="D3" t="n">
-        <v>0.009921641426106284</v>
+        <v>0.1173305580172787</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01482341117047158</v>
+        <v>0.140393589270286</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03449732074526119</v>
+        <v>0.1208409687503152</v>
       </c>
       <c r="G3" t="n">
-        <v>0.03336345081789293</v>
+        <v>0.07725885001891726</v>
       </c>
       <c r="H3" t="n">
-        <v>0.05694890141990666</v>
+        <v>0.1758032892499545</v>
       </c>
     </row>
     <row r="4">
@@ -1913,25 +1913,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1051070761955572</v>
+        <v>0.4196127011536328</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05867705255346009</v>
+        <v>0.3271714169200995</v>
       </c>
       <c r="D4" t="n">
-        <v>0.000213323102649364</v>
+        <v>0.01671054515078844</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0004991518641372274</v>
+        <v>0.03918794839128393</v>
       </c>
       <c r="F4" t="n">
-        <v>0.004095261917459395</v>
+        <v>0.02368996049225053</v>
       </c>
       <c r="G4" t="n">
-        <v>0.004174524373014577</v>
+        <v>0.0135863822458567</v>
       </c>
       <c r="H4" t="n">
-        <v>0.02879439833437964</v>
+        <v>0.1399931590589853</v>
       </c>
     </row>
     <row r="5">
@@ -1941,25 +1941,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.324202214976328</v>
+        <v>0.6477751933762459</v>
       </c>
       <c r="C5" t="n">
-        <v>0.242233467038434</v>
+        <v>0.571989000698527</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01460558463908118</v>
+        <v>0.1292692738077709</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0223417068313329</v>
+        <v>0.197959461484628</v>
       </c>
       <c r="F5" t="n">
-        <v>0.06399423347036352</v>
+        <v>0.1539154329242215</v>
       </c>
       <c r="G5" t="n">
-        <v>0.06461055929965764</v>
+        <v>0.1165606376349096</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1219979610425328</v>
+        <v>0.3029114999877172</v>
       </c>
     </row>
     <row r="6">
@@ -1969,25 +1969,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>27.9240205646043</v>
+        <v>63.32267037234308</v>
       </c>
       <c r="C6" t="n">
-        <v>31.31328864700969</v>
+        <v>53.51522446621205</v>
       </c>
       <c r="D6" t="n">
-        <v>9.305540586436976</v>
+        <v>103.9313656776203</v>
       </c>
       <c r="E6" t="n">
-        <v>27.20068142963095</v>
+        <v>263.3582875568143</v>
       </c>
       <c r="F6" t="n">
-        <v>16.92878018429704</v>
+        <v>39.03103174196716</v>
       </c>
       <c r="G6" t="n">
-        <v>22.79676209996704</v>
+        <v>35.62750364008171</v>
       </c>
       <c r="H6" t="n">
-        <v>22.57817891865767</v>
+        <v>93.13101390917312</v>
       </c>
     </row>
     <row r="7">
@@ -1997,25 +1997,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1422892014881623</v>
+        <v>0.5690604384235899</v>
       </c>
       <c r="C7" t="n">
-        <v>0.08638956849866403</v>
+        <v>0.4811150211226212</v>
       </c>
       <c r="D7" t="n">
-        <v>0.006024340058934072</v>
+        <v>0.7971576998927848</v>
       </c>
       <c r="E7" t="n">
-        <v>0.02361828757270232</v>
+        <v>3.561481421912899</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03277193836230934</v>
+        <v>0.1887918989641253</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03708349492271733</v>
+        <v>0.1224371283961252</v>
       </c>
       <c r="H7" t="n">
-        <v>0.05469613848391491</v>
+        <v>0.9533406014520245</v>
       </c>
     </row>
     <row r="8">
@@ -2025,25 +2025,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-34.29718647753548</v>
+        <v>5.236806734786176</v>
       </c>
       <c r="C8" t="n">
-        <v>-38.53559834178781</v>
+        <v>3.240934479942229</v>
       </c>
       <c r="D8" t="n">
-        <v>-173.506755182954</v>
+        <v>-65.92602156633606</v>
       </c>
       <c r="E8" t="n">
-        <v>-155.6546036028755</v>
+        <v>-48.02710638750537</v>
       </c>
       <c r="F8" t="n">
-        <v>-144.4439642922032</v>
+        <v>-81.0530060697741</v>
       </c>
       <c r="G8" t="n">
-        <v>-132.9688712450058</v>
+        <v>-87.46718233332599</v>
       </c>
       <c r="H8" t="n">
-        <v>-113.234496523727</v>
+        <v>-45.66592919036885</v>
       </c>
     </row>
     <row r="9">
@@ -2053,25 +2053,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-32.63075978942305</v>
+        <v>13.56894017534834</v>
       </c>
       <c r="C9" t="n">
-        <v>-37.11949793958339</v>
+        <v>10.32143649096433</v>
       </c>
       <c r="D9" t="n">
-        <v>-171.4177103075071</v>
+        <v>-55.48079718910184</v>
       </c>
       <c r="E9" t="n">
-        <v>-153.5655587274286</v>
+        <v>-37.58188201027114</v>
       </c>
       <c r="F9" t="n">
-        <v>-141.8522905601945</v>
+        <v>-68.09463740973081</v>
       </c>
       <c r="G9" t="n">
-        <v>-130.5311195952694</v>
+        <v>-75.27842408464399</v>
       </c>
       <c r="H9" t="n">
-        <v>-111.1861561532344</v>
+        <v>-35.42422733790585</v>
       </c>
     </row>
   </sheetData>
@@ -2132,25 +2132,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7388049093520619</v>
+        <v>0.1130861187168157</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8577708012712317</v>
+        <v>0.2033282490118992</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9499652573049657</v>
+        <v>-0.4225667783003679</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7365243664140038</v>
+        <v>-3.377250713582629</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9053226462049749</v>
+        <v>0.4717190389513835</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8715637705300524</v>
+        <v>0.7267780433666391</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8433252918462152</v>
+        <v>-0.3808176736393765</v>
       </c>
     </row>
     <row r="3">
@@ -2160,25 +2160,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1439453803047641</v>
+        <v>0.3405491397571973</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1072821667145773</v>
+        <v>0.2416279038585004</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01683692430117755</v>
+        <v>0.1273807160377483</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02901271390053664</v>
+        <v>0.1134301350595568</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03400282181403558</v>
+        <v>0.1204446634265555</v>
       </c>
       <c r="G3" t="n">
-        <v>0.04258782996654237</v>
+        <v>0.07322022915326605</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0622779728336056</v>
+        <v>0.1694421312154707</v>
       </c>
     </row>
     <row r="4">
@@ -2188,25 +2188,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.121629286498055</v>
+        <v>0.4130043267585664</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05649647661229673</v>
+        <v>0.3164550412268676</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0006568329936611648</v>
+        <v>0.01867479965609344</v>
       </c>
       <c r="E4" t="n">
-        <v>0.001771723762108989</v>
+        <v>0.02943452112216524</v>
       </c>
       <c r="F4" t="n">
-        <v>0.004024132233116191</v>
+        <v>0.02245386418488013</v>
       </c>
       <c r="G4" t="n">
-        <v>0.004850470758028374</v>
+        <v>0.01031839004127341</v>
       </c>
       <c r="H4" t="n">
-        <v>0.03157148714287775</v>
+        <v>0.1350568238316411</v>
       </c>
     </row>
     <row r="5">
@@ -2216,25 +2216,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3487539053516893</v>
+        <v>0.6426541268509574</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2376898748628067</v>
+        <v>0.5625433683076067</v>
       </c>
       <c r="D5" t="n">
-        <v>0.02562875325998448</v>
+        <v>0.136655770665177</v>
       </c>
       <c r="E5" t="n">
-        <v>0.04209184911724584</v>
+        <v>0.1715649180985589</v>
       </c>
       <c r="F5" t="n">
-        <v>0.06343604837248448</v>
+        <v>0.1498461350348421</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0696453211495817</v>
+        <v>0.1015794764766653</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1312076253522987</v>
+        <v>0.2941406325723012</v>
       </c>
     </row>
     <row r="6">
@@ -2244,25 +2244,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>22.40264952955293</v>
+        <v>62.22221744413092</v>
       </c>
       <c r="C6" t="n">
-        <v>28.13007562840134</v>
+        <v>52.07483853457941</v>
       </c>
       <c r="D6" t="n">
-        <v>21.04306862074701</v>
+        <v>109.9823622282129</v>
       </c>
       <c r="E6" t="n">
-        <v>50.4995424251799</v>
+        <v>230.1755335844067</v>
       </c>
       <c r="F6" t="n">
-        <v>16.38709811027314</v>
+        <v>39.48506754799362</v>
       </c>
       <c r="G6" t="n">
-        <v>30.40488573384484</v>
+        <v>72.96655181913506</v>
       </c>
       <c r="H6" t="n">
-        <v>28.14455334133319</v>
+        <v>94.48442852640977</v>
       </c>
     </row>
     <row r="7">
@@ -2272,25 +2272,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1659990277430199</v>
+        <v>0.5606771931159517</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0847162932472382</v>
+        <v>0.4660200541552376</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0179702059040731</v>
+        <v>0.8906847864987517</v>
       </c>
       <c r="E7" t="n">
-        <v>0.08278289670927517</v>
+        <v>2.678558757720609</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03372009870168886</v>
+        <v>0.1797019932440011</v>
       </c>
       <c r="G7" t="n">
-        <v>0.04442619837160415</v>
+        <v>0.09468946001889966</v>
       </c>
       <c r="H7" t="n">
-        <v>0.07160245344614992</v>
+        <v>0.8117220407922418</v>
       </c>
     </row>
     <row r="8">
@@ -2300,25 +2300,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-25.81521742411935</v>
+        <v>6.966947435729205</v>
       </c>
       <c r="C8" t="n">
-        <v>-33.10365505427849</v>
+        <v>4.741388540139084</v>
       </c>
       <c r="D8" t="n">
-        <v>-143.8896961098028</v>
+        <v>-61.59218579475746</v>
       </c>
       <c r="E8" t="n">
-        <v>-123.0518489175913</v>
+        <v>-52.03732921819073</v>
       </c>
       <c r="F8" t="n">
-        <v>-138.9170416115305</v>
+        <v>-80.49989900004995</v>
       </c>
       <c r="G8" t="n">
-        <v>-123.2169878808025</v>
+        <v>-92.34568837127873</v>
       </c>
       <c r="H8" t="n">
-        <v>-97.99907449968748</v>
+        <v>-45.7944610680681</v>
       </c>
     </row>
     <row r="9">
@@ -2328,25 +2328,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-21.64915070383827</v>
+        <v>16.13229422034758</v>
       </c>
       <c r="C9" t="n">
-        <v>-29.56340404876744</v>
+        <v>12.5299407522634</v>
       </c>
       <c r="D9" t="n">
-        <v>-138.6670839211857</v>
+        <v>-50.1024389797998</v>
       </c>
       <c r="E9" t="n">
-        <v>-117.8292367289742</v>
+        <v>-40.54758240323308</v>
       </c>
       <c r="F9" t="n">
-        <v>-132.4378572815089</v>
+        <v>-66.24569347400234</v>
       </c>
       <c r="G9" t="n">
-        <v>-117.1226087564615</v>
+        <v>-78.93805429772851</v>
       </c>
       <c r="H9" t="n">
-        <v>-92.87822357345597</v>
+        <v>-34.52858903035879</v>
       </c>
     </row>
   </sheetData>
@@ -2407,25 +2407,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7736964146988832</v>
+        <v>0.09212463267433868</v>
       </c>
       <c r="C2" t="n">
-        <v>0.858601813513064</v>
+        <v>0.1501112108538304</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9782094616359909</v>
+        <v>-0.4149964112243847</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8889193018310366</v>
+        <v>-4.484551565726319</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9034751457947169</v>
+        <v>0.5198555107245972</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8778047364121809</v>
+        <v>0.6317895762553571</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8801178123143121</v>
+        <v>-0.5842778410737633</v>
       </c>
     </row>
     <row r="3">
@@ -2435,25 +2435,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1372206164809731</v>
+        <v>0.3456196508269823</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1071668293816007</v>
+        <v>0.2602372492759303</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01181013054535976</v>
+        <v>0.1264606903518904</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01863804697535517</v>
+        <v>0.1283459030488752</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03312225494784676</v>
+        <v>0.1119945783097384</v>
       </c>
       <c r="G3" t="n">
-        <v>0.03680084791729295</v>
+        <v>0.07948121999984278</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0574597877080714</v>
+        <v>0.1753565486355432</v>
       </c>
     </row>
     <row r="4">
@@ -2463,25 +2463,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.105381550410637</v>
+        <v>0.4227653470938295</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05616638079438568</v>
+        <v>0.3375939858215468</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0002860561237290228</v>
+        <v>0.01857541937347782</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0007469545087681651</v>
+        <v>0.03688048948305424</v>
       </c>
       <c r="F4" t="n">
-        <v>0.00410265772684419</v>
+        <v>0.02040788888153091</v>
       </c>
       <c r="G4" t="n">
-        <v>0.004614776961674747</v>
+        <v>0.01390568611789188</v>
       </c>
       <c r="H4" t="n">
-        <v>0.02854972942100646</v>
+        <v>0.1416881361285552</v>
       </c>
     </row>
     <row r="5">
@@ -2491,25 +2491,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3246252461079344</v>
+        <v>0.6502040811113304</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2369944741853398</v>
+        <v>0.581028386416315</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01691319377672422</v>
+        <v>0.1362916702277796</v>
       </c>
       <c r="E5" t="n">
-        <v>0.02733046850619588</v>
+        <v>0.1920429365612134</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0640519923721674</v>
+        <v>0.1428561825107017</v>
       </c>
       <c r="G5" t="n">
-        <v>0.06793214969125257</v>
+        <v>0.1179223732711137</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1229745874399357</v>
+        <v>0.3033909383497423</v>
       </c>
     </row>
     <row r="6">
@@ -2519,25 +2519,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>27.91759303961165</v>
+        <v>63.54941805166595</v>
       </c>
       <c r="C6" t="n">
-        <v>30.17874157627624</v>
+        <v>54.40376189025745</v>
       </c>
       <c r="D6" t="n">
-        <v>12.28330468743393</v>
+        <v>110.5248649180972</v>
       </c>
       <c r="E6" t="n">
-        <v>36.47160599518342</v>
+        <v>253.4112200154135</v>
       </c>
       <c r="F6" t="n">
-        <v>18.41352907818878</v>
+        <v>37.97287630262323</v>
       </c>
       <c r="G6" t="n">
-        <v>27.36120425701802</v>
+        <v>37.74504154817007</v>
       </c>
       <c r="H6" t="n">
-        <v>25.43766310561868</v>
+        <v>92.93453045437126</v>
       </c>
     </row>
     <row r="7">
@@ -2547,25 +2547,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1426581608777809</v>
+        <v>0.573798353163379</v>
       </c>
       <c r="C7" t="n">
-        <v>0.08273592250215078</v>
+        <v>0.4967824268189336</v>
       </c>
       <c r="D7" t="n">
-        <v>0.007737400795813055</v>
+        <v>0.8860034338574999</v>
       </c>
       <c r="E7" t="n">
-        <v>0.03484707760682674</v>
+        <v>3.353363624712068</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03282931667037588</v>
+        <v>0.1638288689996925</v>
       </c>
       <c r="G7" t="n">
-        <v>0.04088892294951805</v>
+        <v>0.1256971074059172</v>
       </c>
       <c r="H7" t="n">
-        <v>0.05694946690041091</v>
+        <v>0.9332456358262481</v>
       </c>
     </row>
     <row r="8">
@@ -2575,25 +2575,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-34.25285092956518</v>
+        <v>7.364054189362752</v>
       </c>
       <c r="C8" t="n">
-        <v>-39.19155361377477</v>
+        <v>5.711330036070226</v>
       </c>
       <c r="D8" t="n">
-        <v>-167.3457731212132</v>
+        <v>-61.70423833784939</v>
       </c>
       <c r="E8" t="n">
-        <v>-147.1896317383741</v>
+        <v>-47.30152476935936</v>
       </c>
       <c r="F8" t="n">
-        <v>-144.3952478089421</v>
+        <v>-83.07951106116184</v>
       </c>
       <c r="G8" t="n">
-        <v>-130.4622935298273</v>
+        <v>-84.88643623158755</v>
       </c>
       <c r="H8" t="n">
-        <v>-110.4728917902828</v>
+        <v>-43.98272102908752</v>
       </c>
     </row>
     <row r="9">
@@ -2603,25 +2603,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-32.58642424145275</v>
+        <v>16.52940097398113</v>
       </c>
       <c r="C9" t="n">
-        <v>-37.77545321157035</v>
+        <v>13.49988224819454</v>
       </c>
       <c r="D9" t="n">
-        <v>-165.2567282457664</v>
+        <v>-50.21449152289173</v>
       </c>
       <c r="E9" t="n">
-        <v>-145.1005868629273</v>
+        <v>-35.81177795440171</v>
       </c>
       <c r="F9" t="n">
-        <v>-141.8035740769334</v>
+        <v>-68.82530553511421</v>
       </c>
       <c r="G9" t="n">
-        <v>-128.0245418800909</v>
+        <v>-71.47880215803735</v>
       </c>
       <c r="H9" t="n">
-        <v>-108.4245514197902</v>
+        <v>-32.71684899137822</v>
       </c>
     </row>
   </sheetData>
@@ -2682,25 +2682,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.920063742598861</v>
+        <v>0.726411779233697</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8550242300706042</v>
+        <v>0.7258531696082796</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8915637178429319</v>
+        <v>0.9708809804326931</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7651314696749565</v>
+        <v>0.4674560621939903</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7913946740127938</v>
+        <v>0.9254129066991602</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8751218123077869</v>
+        <v>0.7872243118184897</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8497166077513224</v>
+        <v>0.7672065349977183</v>
       </c>
     </row>
     <row r="3">
@@ -2710,25 +2710,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.09994106982728319</v>
+        <v>0.159877489240433</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1247466765543966</v>
+        <v>0.1490922546980404</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0212527111239967</v>
+        <v>0.009058483378029343</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02253931476548243</v>
+        <v>0.02830952337359156</v>
       </c>
       <c r="F3" t="n">
-        <v>0.05233457662683261</v>
+        <v>0.03279428303835275</v>
       </c>
       <c r="G3" t="n">
-        <v>0.04210461578349364</v>
+        <v>0.05647602664676972</v>
       </c>
       <c r="H3" t="n">
-        <v>0.06048649411358086</v>
+        <v>0.07260134339586945</v>
       </c>
     </row>
     <row r="4">
@@ -2738,25 +2738,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.03722347892874592</v>
+        <v>0.1274003274852153</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05758747337658399</v>
+        <v>0.108896978468517</v>
       </c>
       <c r="D4" t="n">
-        <v>0.00142350143109225</v>
+        <v>0.0003822610403224964</v>
       </c>
       <c r="E4" t="n">
-        <v>0.001579357265356671</v>
+        <v>0.003581055052933547</v>
       </c>
       <c r="F4" t="n">
-        <v>0.008866485834851643</v>
+        <v>0.003170223018443993</v>
       </c>
       <c r="G4" t="n">
-        <v>0.004716099189585667</v>
+        <v>0.008035600685282246</v>
       </c>
       <c r="H4" t="n">
-        <v>0.01856606600436935</v>
+        <v>0.04191107429178575</v>
       </c>
     </row>
     <row r="5">
@@ -2766,25 +2766,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1929338719062724</v>
+        <v>0.3569318247021625</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2399739014488534</v>
+        <v>0.3299954218902393</v>
       </c>
       <c r="D5" t="n">
-        <v>0.03772931792508646</v>
+        <v>0.01955149713762341</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0397411281339203</v>
+        <v>0.05984191718965517</v>
       </c>
       <c r="F5" t="n">
-        <v>0.09416201906741191</v>
+        <v>0.05630473353497016</v>
       </c>
       <c r="G5" t="n">
-        <v>0.06867386103595506</v>
+        <v>0.08964151206490353</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1122023499195833</v>
+        <v>0.1520444844199257</v>
       </c>
     </row>
     <row r="6">
@@ -2794,25 +2794,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>31.56551495638706</v>
+        <v>25.14079915399827</v>
       </c>
       <c r="C6" t="n">
-        <v>42.48157774250674</v>
+        <v>39.74336976680024</v>
       </c>
       <c r="D6" t="n">
-        <v>34.14502427166043</v>
+        <v>13.63992424374445</v>
       </c>
       <c r="E6" t="n">
-        <v>44.10323909287983</v>
+        <v>59.95922179819762</v>
       </c>
       <c r="F6" t="n">
-        <v>31.4921229351972</v>
+        <v>19.29338845990508</v>
       </c>
       <c r="G6" t="n">
-        <v>27.65186461863813</v>
+        <v>35.60052916064681</v>
       </c>
       <c r="H6" t="n">
-        <v>35.23989060287823</v>
+        <v>32.22953876388208</v>
       </c>
     </row>
     <row r="7">
@@ -2822,25 +2822,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.05053731247046384</v>
+        <v>0.1732566954695416</v>
       </c>
       <c r="C7" t="n">
-        <v>0.08430396234242751</v>
+        <v>0.160471934045478</v>
       </c>
       <c r="D7" t="n">
-        <v>0.03402733564888502</v>
+        <v>0.01100328859841782</v>
       </c>
       <c r="E7" t="n">
-        <v>0.07206610918326273</v>
+        <v>0.1642699198788564</v>
       </c>
       <c r="F7" t="n">
-        <v>0.06928813788055802</v>
+        <v>0.02659528410316274</v>
       </c>
       <c r="G7" t="n">
-        <v>0.04126472574037392</v>
+        <v>0.07145762693415067</v>
       </c>
       <c r="H7" t="n">
-        <v>0.05858126387766183</v>
+        <v>0.1011757915049345</v>
       </c>
     </row>
     <row r="8">
@@ -2850,25 +2850,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-53.94386456757291</v>
+        <v>-27.02715641043635</v>
       </c>
       <c r="C8" t="n">
-        <v>-40.8167531654893</v>
+        <v>-25.26029493033172</v>
       </c>
       <c r="D8" t="n">
-        <v>-135.6473485641768</v>
+        <v>-157.2575434532373</v>
       </c>
       <c r="E8" t="n">
-        <v>-133.465483484474</v>
+        <v>-110.2740541037424</v>
       </c>
       <c r="F8" t="n">
-        <v>-125.5878721591766</v>
+        <v>-147.3567402001459</v>
       </c>
       <c r="G8" t="n">
-        <v>-131.9193315990315</v>
+        <v>-112.5968380998875</v>
       </c>
       <c r="H8" t="n">
-        <v>-103.5634422566535</v>
+        <v>-96.62877119963019</v>
       </c>
     </row>
     <row r="9">
@@ -2878,25 +2878,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-53.11065122351669</v>
+        <v>-23.69430303421149</v>
       </c>
       <c r="C9" t="n">
-        <v>-40.10870296438709</v>
+        <v>-22.42809412592288</v>
       </c>
       <c r="D9" t="n">
-        <v>-134.6028261264533</v>
+        <v>-153.0794537023436</v>
       </c>
       <c r="E9" t="n">
-        <v>-132.4209610467505</v>
+        <v>-106.0959643528487</v>
       </c>
       <c r="F9" t="n">
-        <v>-124.2920352931722</v>
+        <v>-142.1733927361285</v>
       </c>
       <c r="G9" t="n">
-        <v>-130.7004557741633</v>
+        <v>-107.7213348004148</v>
       </c>
       <c r="H9" t="n">
-        <v>-102.5392720714072</v>
+        <v>-92.53209045864499</v>
       </c>
     </row>
   </sheetData>
@@ -2957,25 +2957,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9431105538204944</v>
+        <v>0.4204253555122824</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8627538647097533</v>
+        <v>0.4880593710856301</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9731380511535257</v>
+        <v>0.05239166535507711</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9613841049536853</v>
+        <v>-0.1716856824784851</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9021899275116455</v>
+        <v>0.7592406713082724</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8889921836585174</v>
+        <v>0.5314895472077679</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9219281143012702</v>
+        <v>0.3466534879984242</v>
       </c>
     </row>
     <row r="3">
@@ -2985,25 +2985,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.08902164925173872</v>
+        <v>0.2761769702829606</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1123331645170063</v>
+        <v>0.2305937592937447</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01535722088767351</v>
+        <v>0.1067363590841978</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01362723528795824</v>
+        <v>0.07654976174873182</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03428372433901413</v>
+        <v>0.08522472772514221</v>
       </c>
       <c r="G3" t="n">
-        <v>0.02921886286595593</v>
+        <v>0.1000657341971677</v>
       </c>
       <c r="H3" t="n">
-        <v>0.04897364285822448</v>
+        <v>0.1458912187219908</v>
       </c>
     </row>
     <row r="4">
@@ -3013,25 +3013,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0264913966450058</v>
+        <v>0.2698873485965402</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05451709734609628</v>
+        <v>0.203353755957672</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0003526312583227071</v>
+        <v>0.01243976456632939</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0002596699281731947</v>
+        <v>0.007878919720644542</v>
       </c>
       <c r="F4" t="n">
-        <v>0.004157284183036607</v>
+        <v>0.01023314801456466</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0041922763483409</v>
+        <v>0.0176935764968956</v>
       </c>
       <c r="H4" t="n">
-        <v>0.01499505928482925</v>
+        <v>0.08691441889210773</v>
       </c>
     </row>
     <row r="5">
@@ -3041,25 +3041,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1627617788210912</v>
+        <v>0.5195068320980392</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2334889662191691</v>
+        <v>0.4509476199711802</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01877847859446306</v>
+        <v>0.1115336925163396</v>
       </c>
       <c r="E5" t="n">
-        <v>0.01611427715329467</v>
+        <v>0.08876327912287008</v>
       </c>
       <c r="F5" t="n">
-        <v>0.06447700507185959</v>
+        <v>0.1011590233966534</v>
       </c>
       <c r="G5" t="n">
-        <v>0.06474779029697383</v>
+        <v>0.1330172037628802</v>
       </c>
       <c r="H5" t="n">
-        <v>0.09339471602614191</v>
+        <v>0.2341546084779938</v>
       </c>
     </row>
     <row r="6">
@@ -3069,25 +3069,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>24.32232643016287</v>
+        <v>59.27281927258762</v>
       </c>
       <c r="C6" t="n">
-        <v>32.19006526294063</v>
+        <v>48.78328787332875</v>
       </c>
       <c r="D6" t="n">
-        <v>13.81811905620815</v>
+        <v>79.32415761684642</v>
       </c>
       <c r="E6" t="n">
-        <v>14.26791006591968</v>
+        <v>94.58225484610304</v>
       </c>
       <c r="F6" t="n">
-        <v>15.49034871354317</v>
+        <v>33.32517274829666</v>
       </c>
       <c r="G6" t="n">
-        <v>15.54575743996481</v>
+        <v>45.794143357096</v>
       </c>
       <c r="H6" t="n">
-        <v>19.27242116145655</v>
+        <v>60.18030595237641</v>
       </c>
     </row>
     <row r="7">
@@ -3097,25 +3097,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.03661081150535575</v>
+        <v>0.3687935373638934</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0803358087293414</v>
+        <v>0.3019298178446813</v>
       </c>
       <c r="D7" t="n">
-        <v>0.009305426534768187</v>
+        <v>0.2989903355899075</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01276653746361564</v>
+        <v>0.7260418970959935</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03325312067463198</v>
+        <v>0.08539100221771355</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03723693834628342</v>
+        <v>0.1589386393854966</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0349181072089994</v>
+        <v>0.3233475382496143</v>
       </c>
     </row>
     <row r="8">
@@ -3125,25 +3125,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-57.72589931132265</v>
+        <v>1.734239214051453</v>
       </c>
       <c r="C8" t="n">
-        <v>-39.63861370607138</v>
+        <v>0.1078773541429427</v>
       </c>
       <c r="D8" t="n">
-        <v>-162.9518404607099</v>
+        <v>-68.12399946511474</v>
       </c>
       <c r="E8" t="n">
-        <v>-169.3780840501139</v>
+        <v>-77.71485399177863</v>
       </c>
       <c r="F8" t="n">
-        <v>-144.0381179799966</v>
+        <v>-99.717321608769</v>
       </c>
       <c r="G8" t="n">
-        <v>-132.862785283624</v>
+        <v>-76.86384037624885</v>
       </c>
       <c r="H8" t="n">
-        <v>-117.7658901319731</v>
+        <v>-53.42964981228613</v>
       </c>
     </row>
     <row r="9">
@@ -3153,25 +3153,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-56.05947262321022</v>
+        <v>11.73279934272605</v>
       </c>
       <c r="C9" t="n">
-        <v>-38.22251330386696</v>
+        <v>8.604479767369462</v>
       </c>
       <c r="D9" t="n">
-        <v>-160.862795585263</v>
+        <v>-55.58973021243366</v>
       </c>
       <c r="E9" t="n">
-        <v>-167.2890391746671</v>
+        <v>-65.18058473909755</v>
       </c>
       <c r="F9" t="n">
-        <v>-141.446444247988</v>
+        <v>-84.16727921671705</v>
       </c>
       <c r="G9" t="n">
-        <v>-130.4250336338876</v>
+        <v>-62.23733047783044</v>
       </c>
       <c r="H9" t="n">
-        <v>-115.7175497614805</v>
+        <v>-41.13960758933053</v>
       </c>
     </row>
   </sheetData>
@@ -3232,25 +3232,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8019640205902898</v>
+        <v>0.9695101197845015</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8822141585107374</v>
+        <v>0.8581468750836957</v>
       </c>
       <c r="D2" t="n">
-        <v>0.908873563489608</v>
+        <v>0.9693048680841891</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9251973998991592</v>
+        <v>0.9384987207843132</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8806182812863445</v>
+        <v>0.8022037546634957</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8798960873609061</v>
+        <v>0.6611073136951809</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8797939185228408</v>
+        <v>0.8664619420158961</v>
       </c>
     </row>
     <row r="3">
@@ -3260,25 +3260,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1441004245883649</v>
+        <v>0.07231995806291859</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1088601503959113</v>
+        <v>0.1019771427970955</v>
       </c>
       <c r="D3" t="n">
-        <v>0.02372084910291132</v>
+        <v>0.01538470349670535</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01682948735854642</v>
+        <v>0.01439940736048355</v>
       </c>
       <c r="F3" t="n">
-        <v>0.04634280159462015</v>
+        <v>0.08400206074545007</v>
       </c>
       <c r="G3" t="n">
-        <v>0.03154098610558934</v>
+        <v>0.101110126919187</v>
       </c>
       <c r="H3" t="n">
-        <v>0.06189911652432389</v>
+        <v>0.06486556656364001</v>
       </c>
     </row>
     <row r="4">
@@ -3288,25 +3288,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.09221832928327557</v>
+        <v>0.0141980554336714</v>
       </c>
       <c r="C4" t="n">
-        <v>0.04678705285859022</v>
+        <v>0.05634709205877136</v>
       </c>
       <c r="D4" t="n">
-        <v>0.001196265771957996</v>
+        <v>0.0004029515153095287</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0005030049354561645</v>
+        <v>0.0004135611187399137</v>
       </c>
       <c r="F4" t="n">
-        <v>0.005074157684640267</v>
+        <v>0.008407060554007688</v>
       </c>
       <c r="G4" t="n">
-        <v>0.004535795846584166</v>
+        <v>0.01279848428916883</v>
       </c>
       <c r="H4" t="n">
-        <v>0.02505243439675073</v>
+        <v>0.01542786749494479</v>
       </c>
     </row>
     <row r="5">
@@ -3316,25 +3316,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3036747096537273</v>
+        <v>0.1191555933797125</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2163031503667716</v>
+        <v>0.2373754242940312</v>
       </c>
       <c r="D5" t="n">
-        <v>0.03458707521543266</v>
+        <v>0.02007365226632983</v>
       </c>
       <c r="E5" t="n">
-        <v>0.02242777152229273</v>
+        <v>0.02033620217100316</v>
       </c>
       <c r="F5" t="n">
-        <v>0.07123312210369744</v>
+        <v>0.09169002428840167</v>
       </c>
       <c r="G5" t="n">
-        <v>0.06734831732555882</v>
+        <v>0.1131303862327396</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1192623576979134</v>
+        <v>0.1002935471053697</v>
       </c>
     </row>
     <row r="6">
@@ -3344,25 +3344,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36.24222264746874</v>
+        <v>19.67142695695851</v>
       </c>
       <c r="C6" t="n">
-        <v>37.8798940825658</v>
+        <v>24.4297786904916</v>
       </c>
       <c r="D6" t="n">
-        <v>32.65960157139312</v>
+        <v>14.13290174552041</v>
       </c>
       <c r="E6" t="n">
-        <v>29.97016863609783</v>
+        <v>20.35271219204454</v>
       </c>
       <c r="F6" t="n">
-        <v>28.28077476680975</v>
+        <v>30.31799706002684</v>
       </c>
       <c r="G6" t="n">
-        <v>19.90828236020199</v>
+        <v>61.43410228487064</v>
       </c>
       <c r="H6" t="n">
-        <v>30.82349067742287</v>
+        <v>28.38981982165209</v>
       </c>
     </row>
     <row r="7">
@@ -3372,25 +3372,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.124463624321206</v>
+        <v>0.02208560286821952</v>
       </c>
       <c r="C7" t="n">
-        <v>0.06858668944779195</v>
+        <v>0.08499890191603125</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0286753169934882</v>
+        <v>0.01249060563545993</v>
       </c>
       <c r="E7" t="n">
-        <v>0.02329288348507157</v>
+        <v>0.02173987654782399</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03986642599334485</v>
+        <v>0.06822381598875668</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0397062308843371</v>
+        <v>0.1136267448938639</v>
       </c>
       <c r="H7" t="n">
-        <v>0.05409852852087327</v>
+        <v>0.05386092464169254</v>
       </c>
     </row>
     <row r="8">
@@ -3400,25 +3400,25 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-38.52113827316452</v>
+        <v>-60.32905450573071</v>
       </c>
       <c r="C8" t="n">
-        <v>-43.93223143980195</v>
+        <v>-31.14336967228024</v>
       </c>
       <c r="D8" t="n">
-        <v>-139.2995590464668</v>
+        <v>-152.1505805658807</v>
       </c>
       <c r="E8" t="n">
-        <v>-157.4931220933243</v>
+        <v>-151.6048101681858</v>
       </c>
       <c r="F8" t="n">
-        <v>-140.6570580150812</v>
+        <v>-117.0244513692641</v>
       </c>
       <c r="G8" t="n">
-        <v>-132.8938680234089</v>
+        <v>-96.96071324942123</v>
       </c>
       <c r="H8" t="n">
-        <v>-108.7994961485413</v>
+        <v>-101.5354965884604</v>
       </c>
     </row>
     <row r="9">
@@ -3428,25 +3428,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-37.6879249291083</v>
+        <v>-55.32977444139341</v>
       </c>
       <c r="C9" t="n">
-        <v>-43.22418123869974</v>
+        <v>-26.89506846566698</v>
       </c>
       <c r="D9" t="n">
-        <v>-138.2550366087434</v>
+        <v>-145.8834459395401</v>
       </c>
       <c r="E9" t="n">
-        <v>-156.4485996556008</v>
+        <v>-145.3376755418452</v>
       </c>
       <c r="F9" t="n">
-        <v>-139.3612211490769</v>
+        <v>-109.2494301732381</v>
       </c>
       <c r="G9" t="n">
-        <v>-131.6749921985407</v>
+        <v>-89.64745830021204</v>
       </c>
       <c r="H9" t="n">
-        <v>-107.775325963295</v>
+        <v>-95.39047547698264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>